<commit_message>
Report changes and version update in Pom.xml
</commit_message>
<xml_diff>
--- a/ParallelExecution/ExtentResults/TestResultsSummary.xlsx
+++ b/ParallelExecution/ExtentResults/TestResultsSummary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Module Name</t>
   </si>
@@ -43,28 +43,22 @@
     <t>Email Address</t>
   </si>
   <si>
-    <t>C:\PrasanthVB\Selenium_TestNG_ParallelExecution\ParallelExecution\ExtentResults\ExtentReport_Element Test.html</t>
+    <t>C:\PrasanthVB\Selenium_TestNG_ParallelExecution\ParallelExecution\ExtentResults\Admin ExtentReport_Element Test.html</t>
   </si>
   <si>
-    <t>ExtentReport_Element Test.html</t>
+    <t>Admin ExtentReport_Element Test.html</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Element Test</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
+    <t>0</t>
   </si>
 </sst>
 </file>
@@ -134,13 +128,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -186,7 +183,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update TestUtil and pom.xml with latest dependencies
</commit_message>
<xml_diff>
--- a/ParallelExecution/ExtentResults/TestResultsSummary.xlsx
+++ b/ParallelExecution/ExtentResults/TestResultsSummary.xlsx
@@ -107,36 +107,36 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>14</v>
       </c>
     </row>
@@ -151,18 +151,18 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>10</v>
       </c>
     </row>
@@ -177,12 +177,12 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>11</v>
       </c>
     </row>

</xml_diff>